<commit_message>
Itemize Techross quotation by model; add internal item price allocation sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GjFrCobQqqs1TtLcuKd8BA
</commit_message>
<xml_diff>
--- a/내부_마진_정리.xlsx
+++ b/내부_마진_정리.xlsx
@@ -9,7 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="마진 요약" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="매입 구성" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="품목별 견적단가" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="매입 구성" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="71">
   <si>
     <r>
       <rPr>
@@ -498,6 +499,819 @@
     <r>
       <rPr>
         <b val="true"/>
+        <sz val="14"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">품목별 견적 단가 배분  </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">내부용</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="14"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">규칙</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: ① </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">같은 모델은 전 프로젝트 동일 단가  ② </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TSU·ANU CPU = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">프로젝트 타겟  ③ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TM3AQ2 = ANU-S </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 − </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TSU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟  ④ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">모듈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">매입가 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">× (MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">÷ MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">매입 합계</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), 100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원 반올림  ⑤ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MCC CPU = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">나머지</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">프로젝트 타겟</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대 견적가</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">모델</t>
+  </si>
+  <si>
+    <t xml:space="preserve">사용</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수량
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(MCC)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">리스트가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">매입가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">견적 단가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">단가 마진</t>
+  </si>
+  <si>
+    <t xml:space="preserve">배분 방식</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM241C24T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TSU·ANU-S</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TSU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TM241C24R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM241C40T</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ANU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TM241C40R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3AQ2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ANU-S </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 − </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">TSU </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TM241CE40T</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟 − 나머지 모듈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">끝수 조정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF595959"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3DI16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">매입가 비율 배분</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3DQ16T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3DQ8T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3AQ4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3XTRA1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TM3XREC1</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">검증 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대 합계 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF1F3864"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">TSU DC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANU DC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANU-S DC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANU-S AC</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">※ 견적서에 품목 단가가 모두 보이므로</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">같은 견적서 안에서 비교됩니다</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: MCC CPU(TM241CE40T, </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이더넷 포함</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ANU CPU(TM241C40T)</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보다 싸게</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">,</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">    MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아날로그 출력 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4CH(TM3AQ4)</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">가 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ANU-S</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">의 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2CH(TM3AQ2)</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보다 싸게 보입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. MCC </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">타겟</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(1,170,000)</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 다른 프로젝트보다 낮게 잡혀 생기는 현상입니다</t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
         <sz val="13"/>
         <color rgb="FF1F3864"/>
         <rFont val="WenQuanYi Zen Hei"/>
@@ -676,15 +1490,9 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">모델</t>
-  </si>
-  <si>
     <t xml:space="preserve">수량</t>
   </si>
   <si>
-    <t xml:space="preserve">리스트가</t>
-  </si>
-  <si>
     <t xml:space="preserve">할인율</t>
   </si>
   <si>
@@ -694,9 +1502,6 @@
     <t xml:space="preserve">매입 금액</t>
   </si>
   <si>
-    <t xml:space="preserve">TM241C24T</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -720,9 +1525,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">TM241C24R</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -746,9 +1548,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">TM241C40T</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -772,9 +1571,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">TM241C40R</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -798,9 +1594,6 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">TM3AQ2</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b val="true"/>
@@ -845,27 +1638,6 @@
       </rPr>
       <t xml:space="preserve">대 매입가</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">TM241CE40T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TM3DI16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TM3DQ16T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TM3DQ8T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TM3AQ4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TM3XTRA1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TM3XREC1</t>
   </si>
   <si>
     <r>
@@ -901,7 +1673,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1059,15 +1831,15 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="13"/>
-      <color rgb="FF1F3864"/>
+      <sz val="14"/>
+      <color rgb="FFC00000"/>
       <name val="WenQuanYi Zen Hei"/>
       <family val="2"/>
     </font>
     <font>
       <b val="true"/>
-      <sz val="13"/>
-      <color rgb="FF1F3864"/>
+      <sz val="14"/>
+      <color rgb="FFC00000"/>
       <name val="맑은 고딕"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1088,8 +1860,72 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="8"/>
+      <color rgb="FF000000"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF595959"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF595959"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FF1F3864"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF1F3864"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FF375623"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <color rgb="FFC00000"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF1F3864"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
       <color rgb="FF1F3864"/>
       <name val="맑은 고딕"/>
       <family val="0"/>
@@ -1106,7 +1942,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF333333"/>
+        <bgColor rgb="FF333399"/>
       </patternFill>
     </fill>
     <fill>
@@ -1177,7 +2013,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1262,14 +2098,78 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="24" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="24" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1278,23 +2178,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="167" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="25" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="26" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="30" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1375,7 +2267,7 @@
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="FF375623"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -2120,6 +3012,620 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="A1:J29"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>494000</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>646000</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>646000</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>1170000</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="26"/>
+      <c r="D8" s="27" t="n">
+        <v>873000</v>
+      </c>
+      <c r="E8" s="28" t="n">
+        <f aca="false">ROUND(D8*0.4,0)</f>
+        <v>349200</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <f aca="false">$B$5</f>
+        <v>494000</v>
+      </c>
+      <c r="G8" s="28" t="n">
+        <f aca="false">F8-E8</f>
+        <v>144800</v>
+      </c>
+      <c r="H8" s="29" t="n">
+        <f aca="false">IFERROR(G8/F8,0)</f>
+        <v>0.293117408906883</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="26"/>
+      <c r="D9" s="27" t="n">
+        <v>855000</v>
+      </c>
+      <c r="E9" s="28" t="n">
+        <f aca="false">ROUND(D9*0.4,0)</f>
+        <v>342000</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <f aca="false">$B$5</f>
+        <v>494000</v>
+      </c>
+      <c r="G9" s="28" t="n">
+        <f aca="false">F9-E9</f>
+        <v>152000</v>
+      </c>
+      <c r="H9" s="29" t="n">
+        <f aca="false">IFERROR(G9/F9,0)</f>
+        <v>0.307692307692308</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="26"/>
+      <c r="D10" s="27" t="n">
+        <v>928000</v>
+      </c>
+      <c r="E10" s="28" t="n">
+        <f aca="false">ROUND(D10*0.4,0)</f>
+        <v>371200</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <f aca="false">$C$5</f>
+        <v>646000</v>
+      </c>
+      <c r="G10" s="28" t="n">
+        <f aca="false">F10-E10</f>
+        <v>274800</v>
+      </c>
+      <c r="H10" s="29" t="n">
+        <f aca="false">IFERROR(G10/F10,0)</f>
+        <v>0.425386996904025</v>
+      </c>
+      <c r="I10" s="30" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="26"/>
+      <c r="D11" s="27" t="n">
+        <v>903000</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <f aca="false">ROUND(D11*0.4,0)</f>
+        <v>361200</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <f aca="false">$C$5</f>
+        <v>646000</v>
+      </c>
+      <c r="G11" s="28" t="n">
+        <f aca="false">F11-E11</f>
+        <v>284800</v>
+      </c>
+      <c r="H11" s="29" t="n">
+        <f aca="false">IFERROR(G11/F11,0)</f>
+        <v>0.440866873065016</v>
+      </c>
+      <c r="I11" s="30" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="26"/>
+      <c r="D12" s="27" t="n">
+        <v>346000</v>
+      </c>
+      <c r="E12" s="28" t="n">
+        <f aca="false">ROUND(D12*0.35,0)</f>
+        <v>121100</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <f aca="false">$D$5-$B$5</f>
+        <v>152000</v>
+      </c>
+      <c r="G12" s="28" t="n">
+        <f aca="false">F12-E12</f>
+        <v>30900</v>
+      </c>
+      <c r="H12" s="29" t="n">
+        <f aca="false">IFERROR(G12/F12,0)</f>
+        <v>0.203289473684211</v>
+      </c>
+      <c r="I12" s="30" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>920000</v>
+      </c>
+      <c r="E13" s="28" t="n">
+        <f aca="false">ROUND(D13*0.4,0)</f>
+        <v>368000</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <f aca="false">$E$5-SUMPRODUCT($C$14:$C$19,$F$14:$F$19)</f>
+        <v>350800</v>
+      </c>
+      <c r="G13" s="28" t="n">
+        <f aca="false">F13-E13</f>
+        <v>-17200</v>
+      </c>
+      <c r="H13" s="29" t="n">
+        <f aca="false">IFERROR(G13/F13,0)</f>
+        <v>-0.0490307867730901</v>
+      </c>
+      <c r="I13" s="30" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="24" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="27" t="n">
+        <v>228000</v>
+      </c>
+      <c r="E14" s="28" t="n">
+        <f aca="false">ROUND(D14*0.35,0)</f>
+        <v>79800</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <f aca="false">ROUND(E14*($E$5/SUMPRODUCT($C$13:$C$19,$E$13:$E$19)),-2)</f>
+        <v>76100</v>
+      </c>
+      <c r="G14" s="28" t="n">
+        <f aca="false">F14-E14</f>
+        <v>-3700</v>
+      </c>
+      <c r="H14" s="29" t="n">
+        <f aca="false">IFERROR(G14/F14,0)</f>
+        <v>-0.0486202365308804</v>
+      </c>
+      <c r="I14" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>227000</v>
+      </c>
+      <c r="E15" s="28" t="n">
+        <f aca="false">ROUND(D15*0.35,0)</f>
+        <v>79450</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <f aca="false">ROUND(E15*($E$5/SUMPRODUCT($C$13:$C$19,$E$13:$E$19)),-2)</f>
+        <v>75800</v>
+      </c>
+      <c r="G15" s="28" t="n">
+        <f aca="false">F15-E15</f>
+        <v>-3650</v>
+      </c>
+      <c r="H15" s="29" t="n">
+        <f aca="false">IFERROR(G15/F15,0)</f>
+        <v>-0.0481530343007916</v>
+      </c>
+      <c r="I15" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="27" t="n">
+        <v>168000</v>
+      </c>
+      <c r="E16" s="28" t="n">
+        <f aca="false">ROUND(D16*0.35,0)</f>
+        <v>58800</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <f aca="false">ROUND(E16*($E$5/SUMPRODUCT($C$13:$C$19,$E$13:$E$19)),-2)</f>
+        <v>56100</v>
+      </c>
+      <c r="G16" s="28" t="n">
+        <f aca="false">F16-E16</f>
+        <v>-2700</v>
+      </c>
+      <c r="H16" s="29" t="n">
+        <f aca="false">IFERROR(G16/F16,0)</f>
+        <v>-0.0481283422459893</v>
+      </c>
+      <c r="I16" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B17" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>351000</v>
+      </c>
+      <c r="E17" s="28" t="n">
+        <f aca="false">ROUND(D17*0.35,0)</f>
+        <v>122850</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <f aca="false">ROUND(E17*($E$5/SUMPRODUCT($C$13:$C$19,$E$13:$E$19)),-2)</f>
+        <v>117200</v>
+      </c>
+      <c r="G17" s="28" t="n">
+        <f aca="false">F17-E17</f>
+        <v>-5650</v>
+      </c>
+      <c r="H17" s="29" t="n">
+        <f aca="false">IFERROR(G17/F17,0)</f>
+        <v>-0.0482081911262799</v>
+      </c>
+      <c r="I17" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="27" t="n">
+        <v>156000</v>
+      </c>
+      <c r="E18" s="28" t="n">
+        <f aca="false">ROUND(D18*0.35,0)</f>
+        <v>54600</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <f aca="false">ROUND(E18*($E$5/SUMPRODUCT($C$13:$C$19,$E$13:$E$19)),-2)</f>
+        <v>52100</v>
+      </c>
+      <c r="G18" s="28" t="n">
+        <f aca="false">F18-E18</f>
+        <v>-2500</v>
+      </c>
+      <c r="H18" s="29" t="n">
+        <f aca="false">IFERROR(G18/F18,0)</f>
+        <v>-0.0479846449136276</v>
+      </c>
+      <c r="I18" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C19" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="27" t="n">
+        <v>185000</v>
+      </c>
+      <c r="E19" s="28" t="n">
+        <f aca="false">ROUND(D19*0.35,0)</f>
+        <v>64750</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <f aca="false">ROUND(E19*($E$5/SUMPRODUCT($C$13:$C$19,$E$13:$E$19)),-2)</f>
+        <v>61700</v>
+      </c>
+      <c r="G19" s="28" t="n">
+        <f aca="false">F19-E19</f>
+        <v>-3050</v>
+      </c>
+      <c r="H19" s="29" t="n">
+        <f aca="false">IFERROR(G19/F19,0)</f>
+        <v>-0.0494327390599676</v>
+      </c>
+      <c r="I19" s="31" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="32" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="33" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="28" t="n">
+        <f aca="false">F8</f>
+        <v>494000</v>
+      </c>
+      <c r="C22" s="28"/>
+      <c r="D22" s="34" t="str">
+        <f aca="false">IF(F8=$B$5,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="33" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" s="28" t="n">
+        <f aca="false">F10</f>
+        <v>646000</v>
+      </c>
+      <c r="C23" s="28"/>
+      <c r="D23" s="34" t="str">
+        <f aca="false">IF(F10=$C$5,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="28" t="n">
+        <f aca="false">F8+F12</f>
+        <v>646000</v>
+      </c>
+      <c r="C24" s="28"/>
+      <c r="D24" s="34" t="str">
+        <f aca="false">IF(F8+F12=$D$5,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="B25" s="28" t="n">
+        <f aca="false">F9+F12</f>
+        <v>646000</v>
+      </c>
+      <c r="C25" s="28"/>
+      <c r="D25" s="34" t="str">
+        <f aca="false">IF(F9+F12=$D$5,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="28" t="n">
+        <f aca="false">SUMPRODUCT(C13:C19,F13:F19)</f>
+        <v>1170000</v>
+      </c>
+      <c r="C26" s="28"/>
+      <c r="D26" s="34" t="str">
+        <f aca="false">IF(SUMPRODUCT(C13:C19,F13:F19)=$E$5,"일치","불일치")</f>
+        <v>일치</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="35" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="35"/>
+      <c r="C28" s="35"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="35"/>
+      <c r="F28" s="35"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="35"/>
+      <c r="I28" s="35"/>
+      <c r="J28" s="35"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="36" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" s="36"/>
+      <c r="C29" s="36"/>
+      <c r="D29" s="36"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="36"/>
+      <c r="I29" s="36"/>
+      <c r="J29" s="36"/>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A29:J29"/>
+  </mergeCells>
+  <conditionalFormatting sqref="G8:H19">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>G8&lt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1:H32"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -2133,569 +3639,569 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="A1" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="38" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="21" t="s">
+      <c r="C4" s="38" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="21" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="21" t="s">
+      <c r="D4" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="E4" s="38" t="s">
         <v>28</v>
       </c>
+      <c r="F4" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="G4" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="38" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="33" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" s="24" t="n">
+      <c r="C5" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="25" t="n">
+      <c r="E5" s="27" t="n">
         <v>873000</v>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="41" t="n">
         <v>0.4</v>
       </c>
-      <c r="G5" s="27" t="n">
+      <c r="G5" s="28" t="n">
         <f aca="false">ROUND(E5*F5,0)</f>
         <v>349200</v>
       </c>
-      <c r="H5" s="27" t="n">
+      <c r="H5" s="28" t="n">
         <f aca="false">D5*G5</f>
         <v>349200</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="28"/>
-      <c r="C6" s="28"/>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="29" t="n">
+      <c r="A6" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="42"/>
+      <c r="F6" s="42"/>
+      <c r="G6" s="42"/>
+      <c r="H6" s="43" t="n">
         <f aca="false">SUM(H5:H5)</f>
         <v>349200</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="33" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="24" t="n">
+      <c r="C8" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="27" t="n">
         <v>855000</v>
       </c>
-      <c r="F8" s="26" t="n">
+      <c r="F8" s="41" t="n">
         <v>0.4</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="28" t="n">
         <f aca="false">ROUND(E8*F8,0)</f>
         <v>342000</v>
       </c>
-      <c r="H8" s="27" t="n">
+      <c r="H8" s="28" t="n">
         <f aca="false">D8*G8</f>
         <v>342000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
-      <c r="D9" s="28"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="28"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="29" t="n">
+      <c r="A9" s="42" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="42"/>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
+      <c r="E9" s="42"/>
+      <c r="F9" s="42"/>
+      <c r="G9" s="42"/>
+      <c r="H9" s="43" t="n">
         <f aca="false">SUM(H8:H8)</f>
         <v>342000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="33" t="s">
         <v>15</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="24" t="n">
+      <c r="C11" s="39" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="25" t="n">
+      <c r="E11" s="27" t="n">
         <v>928000</v>
       </c>
-      <c r="F11" s="26" t="n">
+      <c r="F11" s="41" t="n">
         <v>0.4</v>
       </c>
-      <c r="G11" s="27" t="n">
+      <c r="G11" s="28" t="n">
         <f aca="false">ROUND(E11*F11,0)</f>
         <v>371200</v>
       </c>
-      <c r="H11" s="27" t="n">
+      <c r="H11" s="28" t="n">
         <f aca="false">D11*G11</f>
         <v>371200</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="28" t="s">
-        <v>34</v>
-      </c>
-      <c r="B12" s="28"/>
-      <c r="C12" s="28"/>
-      <c r="D12" s="28"/>
-      <c r="E12" s="28"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="28"/>
-      <c r="H12" s="29" t="n">
+      <c r="A12" s="42" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="43" t="n">
         <f aca="false">SUM(H11:H11)</f>
         <v>371200</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="33" t="s">
         <v>15</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="24" t="n">
+      <c r="C14" s="39" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E14" s="27" t="n">
         <v>903000</v>
       </c>
-      <c r="F14" s="26" t="n">
+      <c r="F14" s="41" t="n">
         <v>0.4</v>
       </c>
-      <c r="G14" s="27" t="n">
+      <c r="G14" s="28" t="n">
         <f aca="false">ROUND(E14*F14,0)</f>
         <v>361200</v>
       </c>
-      <c r="H14" s="27" t="n">
+      <c r="H14" s="28" t="n">
         <f aca="false">D14*G14</f>
         <v>361200</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="29" t="n">
+      <c r="A15" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="42"/>
+      <c r="G15" s="42"/>
+      <c r="H15" s="43" t="n">
         <f aca="false">SUM(H14:H14)</f>
         <v>361200</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C17" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="D17" s="24" t="n">
+      <c r="C17" s="39" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="27" t="n">
         <v>873000</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="41" t="n">
         <v>0.4</v>
       </c>
-      <c r="G17" s="27" t="n">
+      <c r="G17" s="28" t="n">
         <f aca="false">ROUND(E17*F17,0)</f>
         <v>349200</v>
       </c>
-      <c r="H17" s="27" t="n">
+      <c r="H17" s="28" t="n">
         <f aca="false">D17*G17</f>
         <v>349200</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C18" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="24" t="n">
+      <c r="C18" s="39" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="25" t="n">
+      <c r="E18" s="27" t="n">
         <v>346000</v>
       </c>
-      <c r="F18" s="26" t="n">
+      <c r="F18" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G18" s="27" t="n">
+      <c r="G18" s="28" t="n">
         <f aca="false">ROUND(E18*F18,0)</f>
         <v>121100</v>
       </c>
-      <c r="H18" s="27" t="n">
+      <c r="H18" s="28" t="n">
         <f aca="false">D18*G18</f>
         <v>121100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="B19" s="28"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-      <c r="F19" s="28"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="29" t="n">
+      <c r="A19" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="42"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="42"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="42"/>
+      <c r="G19" s="42"/>
+      <c r="H19" s="43" t="n">
         <f aca="false">SUM(H17:H18)</f>
         <v>470300</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C21" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="24" t="n">
+      <c r="C21" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="25" t="n">
+      <c r="E21" s="27" t="n">
         <v>855000</v>
       </c>
-      <c r="F21" s="26" t="n">
+      <c r="F21" s="41" t="n">
         <v>0.4</v>
       </c>
-      <c r="G21" s="27" t="n">
+      <c r="G21" s="28" t="n">
         <f aca="false">ROUND(E21*F21,0)</f>
         <v>342000</v>
       </c>
-      <c r="H21" s="27" t="n">
+      <c r="H21" s="28" t="n">
         <f aca="false">D21*G21</f>
         <v>342000</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="33" t="s">
         <v>16</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C22" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="D22" s="24" t="n">
+      <c r="C22" s="39" t="s">
+        <v>40</v>
+      </c>
+      <c r="D22" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="25" t="n">
+      <c r="E22" s="27" t="n">
         <v>346000</v>
       </c>
-      <c r="F22" s="26" t="n">
+      <c r="F22" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G22" s="27" t="n">
+      <c r="G22" s="28" t="n">
         <f aca="false">ROUND(E22*F22,0)</f>
         <v>121100</v>
       </c>
-      <c r="H22" s="27" t="n">
+      <c r="H22" s="28" t="n">
         <f aca="false">D22*G22</f>
         <v>121100</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="28" t="s">
-        <v>39</v>
-      </c>
-      <c r="B23" s="28"/>
-      <c r="C23" s="28"/>
-      <c r="D23" s="28"/>
-      <c r="E23" s="28"/>
-      <c r="F23" s="28"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="29" t="n">
+      <c r="A23" s="42" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" s="42"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="43" t="n">
         <f aca="false">SUM(H21:H22)</f>
         <v>463100</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="24" t="n">
+      <c r="C25" s="39" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="25" t="n">
+      <c r="E25" s="27" t="n">
         <v>920000</v>
       </c>
-      <c r="F25" s="26" t="n">
+      <c r="F25" s="41" t="n">
         <v>0.4</v>
       </c>
-      <c r="G25" s="27" t="n">
+      <c r="G25" s="28" t="n">
         <f aca="false">ROUND(E25*F25,0)</f>
         <v>368000</v>
       </c>
-      <c r="H25" s="27" t="n">
+      <c r="H25" s="28" t="n">
         <f aca="false">D25*G25</f>
         <v>368000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="23" t="s">
-        <v>41</v>
-      </c>
-      <c r="D26" s="24" t="n">
+      <c r="C26" s="39" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="40" t="n">
         <v>5</v>
       </c>
-      <c r="E26" s="25" t="n">
+      <c r="E26" s="27" t="n">
         <v>228000</v>
       </c>
-      <c r="F26" s="26" t="n">
+      <c r="F26" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G26" s="27" t="n">
+      <c r="G26" s="28" t="n">
         <f aca="false">ROUND(E26*F26,0)</f>
         <v>79800</v>
       </c>
-      <c r="H26" s="27" t="n">
+      <c r="H26" s="28" t="n">
         <f aca="false">D26*G26</f>
         <v>399000</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C27" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="D27" s="24" t="n">
+      <c r="C27" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="25" t="n">
+      <c r="E27" s="27" t="n">
         <v>227000</v>
       </c>
-      <c r="F27" s="26" t="n">
+      <c r="F27" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G27" s="27" t="n">
+      <c r="G27" s="28" t="n">
         <f aca="false">ROUND(E27*F27,0)</f>
         <v>79450</v>
       </c>
-      <c r="H27" s="27" t="n">
+      <c r="H27" s="28" t="n">
         <f aca="false">D27*G27</f>
         <v>158900</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C28" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D28" s="24" t="n">
+      <c r="C28" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="25" t="n">
+      <c r="E28" s="27" t="n">
         <v>168000</v>
       </c>
-      <c r="F28" s="26" t="n">
+      <c r="F28" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G28" s="27" t="n">
+      <c r="G28" s="28" t="n">
         <f aca="false">ROUND(E28*F28,0)</f>
         <v>58800</v>
       </c>
-      <c r="H28" s="27" t="n">
+      <c r="H28" s="28" t="n">
         <f aca="false">D28*G28</f>
         <v>58800</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" s="24" t="n">
+      <c r="C29" s="39" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="25" t="n">
+      <c r="E29" s="27" t="n">
         <v>351000</v>
       </c>
-      <c r="F29" s="26" t="n">
+      <c r="F29" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G29" s="27" t="n">
+      <c r="G29" s="28" t="n">
         <f aca="false">ROUND(E29*F29,0)</f>
         <v>122850</v>
       </c>
-      <c r="H29" s="27" t="n">
+      <c r="H29" s="28" t="n">
         <f aca="false">D29*G29</f>
         <v>122850</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C30" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="D30" s="24" t="n">
+      <c r="C30" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="D30" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="25" t="n">
+      <c r="E30" s="27" t="n">
         <v>156000</v>
       </c>
-      <c r="F30" s="26" t="n">
+      <c r="F30" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G30" s="27" t="n">
+      <c r="G30" s="28" t="n">
         <f aca="false">ROUND(E30*F30,0)</f>
         <v>54600</v>
       </c>
-      <c r="H30" s="27" t="n">
+      <c r="H30" s="28" t="n">
         <f aca="false">D30*G30</f>
         <v>54600</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="33" t="s">
         <v>17</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C31" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="D31" s="24" t="n">
+      <c r="C31" s="39" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="25" t="n">
+      <c r="E31" s="27" t="n">
         <v>185000</v>
       </c>
-      <c r="F31" s="26" t="n">
+      <c r="F31" s="41" t="n">
         <v>0.35</v>
       </c>
-      <c r="G31" s="27" t="n">
+      <c r="G31" s="28" t="n">
         <f aca="false">ROUND(E31*F31,0)</f>
         <v>64750</v>
       </c>
-      <c r="H31" s="27" t="n">
+      <c r="H31" s="28" t="n">
         <f aca="false">D31*G31</f>
         <v>64750</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="28" t="s">
-        <v>47</v>
-      </c>
-      <c r="B32" s="28"/>
-      <c r="C32" s="28"/>
-      <c r="D32" s="28"/>
-      <c r="E32" s="28"/>
-      <c r="F32" s="28"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="29" t="n">
+      <c r="A32" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="B32" s="42"/>
+      <c r="C32" s="42"/>
+      <c r="D32" s="42"/>
+      <c r="E32" s="42"/>
+      <c r="F32" s="42"/>
+      <c r="G32" s="42"/>
+      <c r="H32" s="43" t="n">
         <f aca="false">SUM(H25:H31)</f>
         <v>1226900</v>
       </c>

</xml_diff>